<commit_message>
Update project files and configurations
</commit_message>
<xml_diff>
--- a/data/raw/구분상가매매.xlsx
+++ b/data/raw/구분상가매매.xlsx
@@ -2343,7 +2343,7 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
@@ -2701,7 +2701,7 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
@@ -2797,7 +2797,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
@@ -2893,7 +2893,7 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
@@ -2993,7 +2993,7 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="P28" t="inlineStr">
@@ -4061,7 +4061,7 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="P39" t="inlineStr">
@@ -4743,12 +4743,12 @@
       <c r="N46" t="inlineStr"/>
       <c r="O46" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="P46" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>4.90%</t>
         </is>
       </c>
       <c r="Q46" t="inlineStr">
@@ -5039,7 +5039,7 @@
       <c r="N49" t="inlineStr"/>
       <c r="O49" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="P49" t="inlineStr">
@@ -5922,7 +5922,7 @@
       </c>
       <c r="P58" t="inlineStr">
         <is>
-          <t>4.90%</t>
+          <t>5%</t>
         </is>
       </c>
       <c r="Q58" t="inlineStr"/>
@@ -6012,7 +6012,7 @@
       </c>
       <c r="P59" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>4.90%</t>
         </is>
       </c>
       <c r="Q59" t="inlineStr">
@@ -6201,7 +6201,7 @@
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="P61" t="inlineStr">
@@ -6571,7 +6571,7 @@
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="P65" t="inlineStr">
@@ -7067,7 +7067,7 @@
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="P70" t="inlineStr">
@@ -7175,7 +7175,7 @@
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="P71" t="inlineStr">
@@ -7366,7 +7366,7 @@
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="P73" t="inlineStr">
@@ -7474,7 +7474,7 @@
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="P74" t="inlineStr">
@@ -7772,7 +7772,7 @@
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="P77" t="inlineStr">
@@ -7885,7 +7885,7 @@
       </c>
       <c r="P78" t="inlineStr">
         <is>
-          <t>4.90%</t>
+          <t>5%</t>
         </is>
       </c>
       <c r="Q78" t="inlineStr">
@@ -8158,7 +8158,7 @@
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="P81" t="inlineStr">
@@ -9034,7 +9034,7 @@
       </c>
       <c r="O90" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="P90" t="inlineStr">
@@ -9746,7 +9746,7 @@
       </c>
       <c r="O97" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="P97" t="inlineStr">
@@ -9954,7 +9954,7 @@
       <c r="N99" t="inlineStr"/>
       <c r="O99" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="P99" t="inlineStr">
@@ -10148,7 +10148,7 @@
       </c>
       <c r="O101" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="P101" t="inlineStr">
@@ -10234,7 +10234,7 @@
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="P102" t="inlineStr">
@@ -10326,7 +10326,7 @@
       <c r="N103" t="inlineStr"/>
       <c r="O103" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="P103" t="inlineStr">
@@ -10508,7 +10508,7 @@
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="P105" t="inlineStr">
@@ -11538,7 +11538,7 @@
       <c r="N117" t="inlineStr"/>
       <c r="O117" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="P117" t="inlineStr">
@@ -11626,7 +11626,7 @@
       <c r="N118" t="inlineStr"/>
       <c r="O118" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="P118" t="inlineStr">
@@ -11898,7 +11898,7 @@
       <c r="N121" t="inlineStr"/>
       <c r="O121" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="P121" t="inlineStr">
@@ -12246,7 +12246,7 @@
       <c r="N125" t="inlineStr"/>
       <c r="O125" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="P125" t="inlineStr">
@@ -12346,7 +12346,7 @@
       </c>
       <c r="O126" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="P126" t="inlineStr">
@@ -12620,7 +12620,7 @@
       <c r="N129" t="inlineStr"/>
       <c r="O129" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="P129" t="inlineStr">
@@ -12906,7 +12906,7 @@
       <c r="N132" t="inlineStr"/>
       <c r="O132" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="P132" t="inlineStr">
@@ -13006,7 +13006,7 @@
       <c r="N133" t="inlineStr"/>
       <c r="O133" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="P133" t="inlineStr">
@@ -13586,7 +13586,7 @@
       <c r="N139" t="inlineStr"/>
       <c r="O139" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="P139" t="inlineStr">
@@ -14239,7 +14239,7 @@
       </c>
       <c r="O146" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="P146" t="inlineStr">
@@ -14599,7 +14599,7 @@
       <c r="N150" t="inlineStr"/>
       <c r="O150" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="P150" t="inlineStr">
@@ -14901,7 +14901,7 @@
       </c>
       <c r="O153" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="P153" t="inlineStr">
@@ -15001,7 +15001,7 @@
       </c>
       <c r="O154" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="P154" t="inlineStr">
@@ -15205,7 +15205,7 @@
       </c>
       <c r="O156" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="P156" t="inlineStr">
@@ -15826,7 +15826,7 @@
       </c>
       <c r="P162" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>4.90%</t>
         </is>
       </c>
       <c r="Q162" t="inlineStr">
@@ -15921,7 +15921,7 @@
       </c>
       <c r="O163" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="P163" t="inlineStr">
@@ -16025,7 +16025,7 @@
       </c>
       <c r="O164" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="P164" t="inlineStr">
@@ -16390,7 +16390,7 @@
       </c>
       <c r="O168" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="P168" t="inlineStr">
@@ -16478,7 +16478,7 @@
       </c>
       <c r="O169" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="P169" t="inlineStr">
@@ -16566,7 +16566,7 @@
       </c>
       <c r="O170" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="P170" t="inlineStr">
@@ -16814,7 +16814,7 @@
       <c r="N173" t="inlineStr"/>
       <c r="O173" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="P173" t="inlineStr">
@@ -16914,7 +16914,7 @@
       </c>
       <c r="O174" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="P174" t="inlineStr">
@@ -17733,7 +17733,7 @@
       </c>
       <c r="N182" t="inlineStr">
         <is>
-          <t>1400</t>
+          <t>1400.00</t>
         </is>
       </c>
       <c r="O182" t="inlineStr">
@@ -18047,7 +18047,7 @@
       </c>
       <c r="O185" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="P185" t="inlineStr">
@@ -18364,7 +18364,7 @@
       <c r="N188" t="inlineStr"/>
       <c r="O188" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="P188" t="inlineStr">
@@ -18649,7 +18649,7 @@
       <c r="N191" t="inlineStr"/>
       <c r="O191" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="P191" t="inlineStr">
@@ -19649,7 +19649,7 @@
       <c r="N202" t="inlineStr"/>
       <c r="O202" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="P202" t="inlineStr">
@@ -19749,7 +19749,7 @@
       </c>
       <c r="O203" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="P203" t="inlineStr">
@@ -19883,7 +19883,7 @@
       <c r="N205" t="inlineStr"/>
       <c r="O205" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="P205" t="inlineStr">
@@ -19981,7 +19981,7 @@
       </c>
       <c r="O206" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="P206" t="inlineStr">
@@ -20259,7 +20259,7 @@
       <c r="N209" t="inlineStr"/>
       <c r="O209" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="P209" t="inlineStr">
@@ -21107,7 +21107,7 @@
       </c>
       <c r="O218" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="P218" t="inlineStr">
@@ -21211,7 +21211,7 @@
       <c r="N219" t="inlineStr"/>
       <c r="O219" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="P219" t="inlineStr">
@@ -21495,7 +21495,7 @@
       <c r="N222" t="inlineStr"/>
       <c r="O222" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="P222" t="inlineStr">
@@ -21556,7 +21556,7 @@
       </c>
       <c r="P223" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>4.50%</t>
         </is>
       </c>
       <c r="Q223" t="inlineStr"/>
@@ -67381,7 +67381,7 @@
       <c r="N2128" t="inlineStr"/>
       <c r="O2128" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="P2128" t="inlineStr">
@@ -67509,7 +67509,7 @@
       <c r="N2132" t="inlineStr"/>
       <c r="O2132" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="P2132" t="inlineStr">
@@ -67541,7 +67541,7 @@
       <c r="N2133" t="inlineStr"/>
       <c r="O2133" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="P2133" t="inlineStr">
@@ -67578,7 +67578,7 @@
       </c>
       <c r="P2134" t="inlineStr">
         <is>
-          <t>3.50%</t>
+          <t>4%</t>
         </is>
       </c>
       <c r="Q2134" t="inlineStr"/>
@@ -67669,7 +67669,7 @@
       <c r="N2137" t="inlineStr"/>
       <c r="O2137" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="P2137" t="inlineStr">
@@ -67705,7 +67705,7 @@
       <c r="N2138" t="inlineStr"/>
       <c r="O2138" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="P2138" t="inlineStr">

</xml_diff>